<commit_message>
chore: add planning docs, test-reports tooling, xlsx generators
- docs: add e2e-plan and superpowers specs/plans for file-upload endpoints
  and whitelabel→branding rename
- scripts: replace generate_clients_e2e with build_xlsx + build_employees_tests
- test-reports: add README for the HTML report pipeline
- root: update package.json, package-lock.json, e2e_test_clients.xlsx,
  Arabic test inventory doc
- dashboard: include remaining branches-edit e2e tweaks

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e_test_clients.xlsx
+++ b/e2e_test_clients.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="E2E Test Cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="E2E Employees" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'E2E Test Cases'!$A$1:$P$1</definedName>
@@ -66,7 +67,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +84,20 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -106,11 +119,25 @@
         <color rgb="00B4B4B4"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,6 +156,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6254,4 +6293,2354 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case Title</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Executed By</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Execution Date</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Defect ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="80" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>EM-001</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>عرض قائمة الممارسين</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>جلب قائمة الممارسين مع pagination و stats</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>1. مستخدم مسجّل دخول
+2. وجود ممارسين في التينانت</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح /employees
+2. لاحظ StatsGrid + الجدول</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>page=1&amp;limit=20</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
+        <is>
+          <t>1. GET /dashboard/people/employees → 200
+2. GET /dashboard/people/employees/stats → 200
+3. الكروت: الإجمالي/نشط/غير متاح/متوسط التقييم
+4. الجدول يعرض الممارسين</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>نجح: القائمة + stats يُحمَّلان من endpoints منفصلة. stats لا تتأثر بالفلاتر.</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr"/>
+    </row>
+    <row r="3" ht="80" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>EM-002</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>بحث Debounce</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>البحث في القائمة بـ debounce 300ms</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>قائمة غير فارغة</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>1. اكتب 5 أحرف سريعة في حقل البحث</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>search=tariq</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>طلب واحد فقط بعد 300ms (ليس طلب لكل حرف)</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>نجح: قبل الإصلاح كان 5 طلبات، الآن طلب واحد.</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: use-employees.ts — useEffect + setTimeout 300ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>EM-003</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>فلتر الحالة isActive</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>فلترة الممارسين بـ isActive=false عبر combobox</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>ممارس نشط + ممارس معطّل</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح combobox (جميع الحالات)
+2. اختر (غير متاح)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>isActive=false</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>1. GET ?isActive=false → 200
+2. عرض المعطّلين فقط
+3. Stats لا تتأثر بالفلتر</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: الباك كان يتجاهل الفلتر بسبب ValidationPipe implicit conversion. الحل: parse يدوي في الـ controller.</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: people.controller.ts — @Query(isActive) rawIsActive</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>EM-004</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Stats endpoint</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>الإحصائيات مستقلة عن فلاتر القائمة</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>ممارسون بحالات متنوعة</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>1. ابحث عن اسم غير موجود
+2. لاحظ StatsGrid</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>search=zzznotfound</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>الجدول فارغ، لكن Stats تظل تعرض total/active الكلي</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>نجح: أُضيف GET /employees/stats جديد يحسب total/active/inactive/avgRating بدون فلاتر.</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Added: employee-stats.handler.ts + useEmployeeStats hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>EM-010</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>إنشاء ممارس (Tab 1: Basic Info)</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>ملء المعلومات الأساسية وإرسال onboarding</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>مستخدم بصلاحية إنشاء</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط (إضافة ممارس)
+2. املأ: اللقب، البريد، الاسم AR+EN، التخصص AR+EN، الخبرة، التعليم، النبذة</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>title=دكتور
+nameEn=Dr. Ahmed
+nameAr=د. أحمد
+email=dr.ahmed@test.com
+specialty=Dermatologist
+experience=8</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>1. POST /employees/onboarding → 201
+2. جميع الحقول تُرسل في الـ payload
+3. الرد يحتوي employee.id</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>نجح: كل الحقول محفوظة بشكل صحيح. payload نظيف.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>EM-011</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>إنشاء ممارس (Tab 2: Schedule)</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>تحديد أيام العمل وتفعيل/تعطيل أيام</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Tab 1 مملوء</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>1. انتقل لتاب (الجدول والاستراحات)
+2. عطّل الخميس
+3. فعّل السبت
+4. أضف استراحة للاثنين</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>days: Sun/Mon/Tue/Wed + Sat
+break: Monday 12:00-13:00</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>PATCH /employees/:id/availability → 200
+body.windows يحتوي 6 أيام (0,1,2,3,6 بدون 4 و 5)</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>نجح: windows محفوظة بالـ dayOfWeek الصحيح.</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>EM-012</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Breaks endpoint مفقود</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>الاستراحات يفترض أن تُرسل لـ PUT /breaks لكن endpoint مفقود</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>استراحة مُضافة في الفورم</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>1. املأ استراحة للاثنين
+2. احفظ الممارس</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>breaks: [{dayOfWeek:1, startTime:12:00, endTime:13:00}]</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>PUT /employees/:id/breaks → 200</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>فشل قبل الإصلاح: 404. بعد الإصلاح: أُضيف PUT stub يعيد 200 (no-op حتى migration split-shifts).</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: people.controller.ts — PUT /breaks stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>EM-013</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>إنشاء ممارس (Tab 3: Services)</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>ربط خدمة بسعر ومدة مختلفين لكل نوع حجز</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>خدمة موجودة في النظام</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>1. انتقل لتاب (الخدمات والتسعير)
+2. اختر خدمة
+3. حضوري: 300 ر.س / 45 دق
+4. عن بُعد: 200 ر.س / 30 دق
+5. buffer: 15 دق</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>in_person: 300/45
+online: 200/30
+buffer: 15</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>POST /employees/:id/services → 201
+payload يحتوي types[] + bufferMinutes</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جزئي: POST 201، لكن الباك يتجاهل price/duration/types (Schema EmployeeService فقيرة). يحتاج migration.</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>P0-Critical</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>BUG: assign-employee-service.handler يتجاهل التسعير. Schema تحتاج حقول جديدة + EmployeeServiceType model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>EM-014</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Dropdown الخدمات — ??? ???</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>خدمة بـ nameAr null تظهر كـ ??? ???</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>خدمة في DB بـ nameAr فارغ</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح dropdown الخدمات في tab 3</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>تجاهل الخدمات بدون اسم أو استخدام fallback</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: تجاهل الخدمات بدون اسم، fallback بين AR/EN.</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>P3-Low</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: add-service-form.tsx + assign-service-sheet.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>EM-015</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>CREATE — القائمة تُحدَّث بعد الإنشاء</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>السجل الجديد يظهر بدون reload يدوي</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>ممارس تم إنشاؤه للتو</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>1. أنشئ ممارس جديد
+2. بعد redirect لـ /employees
+3. لاحظ الجدول</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>السجل الجديد يظهر + stats تحدّث</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: أُضيف refetchType:all للـ invalidate.</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: use-employee-mutations.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>EM-020</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>صفحة التفاصيل</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>عرض بيانات الممارس بعد الإنشاء</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>ممارس موجود</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط (معاينة) في صف الجدول
+2. لاحظ صفحة detail</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>1. GET /employees/:id → 200
+2. عرض: الاسم، التخصص، الخبرة، التعليم، النبذة، أوقات العمل، الخدمات
+3. روابط (تعديل)</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد إصلاح bugs: list-employee-services ما كان يحمّل service relation. الآن يحمّل يدوياً.</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: list-employee-services.handler.ts + employee-services-section.tsx null-safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>EM-021</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Preview button</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>زر المعاينة ينتقل لصفحة التفاصيل</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>صف ممارس في الجدول</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط أيقونة العين</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>الانتقال لـ /employees/:id</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: aria-label كان common.preview (خام)، الآن معاينة وcallback مربوط.</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: ar.nav.ts + en.nav.ts — common.preview key</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>EM-030</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>تعديل المعلومات الأساسية</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>تغيير اللقب والخبرة وحفظ</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>ممارس موجود</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط (تعديل)
+2. غيّر اللقب لـ بروفيسور
+3. غيّر الخبرة لـ 15
+4. احفظ</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>title=بروفيسور
+experience=15</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>1. PATCH /employees/:id → 200
+2. Toast نجاح
+3. Redirect إلى /employees
+4. القائمة تعرض 15 سنة</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>نجح: الحقول محفوظة. القائمة تحدّثت بعد invalidation.</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>EM-031</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>EDIT — side effects block redirect</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>فشل side effect (breaks 404) يمنع toast/redirect</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>ممارس مع استراحات</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح تعديل
+2. غيّر شيء
+3. احفظ</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>حتى لو فشل PUT /breaks، الـ PATCH الأساسي ينجح ويعرض toast + redirect</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: Side effects في try/catch منفصلة، الأخطاء تُجمع كـ warning لكن الـ redirect يحدث.</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: use-employee-form.ts — submitEdit refactored</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>EM-032</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>EDIT — invalidate list</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>التعديل ينعكس في القائمة</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>ممارس معدّل</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>1. عدّل ممارس
+2. ارجع لـ /employees</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>القائمة تعرض القيم الجديدة بدون reload</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: refetchType:all يُجبر refetch.</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>EM-040</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>حذف ممارس</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>حذف ممارس مع تأكيد</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>ممارس موجود</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط أيقونة الحذف
+2. confirmation dialog
+3. اضغط (حذف)</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>1. DELETE /employees/:id → 204
+2. Toast نجاح
+3. اختفاء من القائمة
+4. Stats تحدّث من 1→0</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: كان stub يعرض toast.error فقط. الآن mutation حقيقية + invalidate stats + handle 204.</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>P0-Critical</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: delete-employee-dialog.tsx + api.ts (handle 204 No Content)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>EM-041</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>DELETE — إلغاء التأكيد</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>ضغط إلغاء لا يحذف</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Dialog مفتوح</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط (إلغاء)</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>1. Dialog يُغلق
+2. لا طلب DELETE
+3. السجل موجود</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>نجح.</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>EM-050</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>إضافة إجازة</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>تفعيل الإجازة في EDIT مع تواريخ</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>ممارس في صفحة EDIT</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>1. فعّل switch الإجازة
+2. حدد تاريخ بداية/نهاية
+3. احفظ</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>startDate=2026-05-01
+endDate=2026-05-10</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>POST /employees/:id/vacations → 201</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: endpoint كان 404، أُضيف alias للـ exceptions.</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t>Added: POST/GET/DELETE /employees/:id/vacations</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>EM-051</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>عرض الإجازات القادمة</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>detail page تعرض الإجازات</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>ممارس له إجازة</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح detail</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>GET /employees/:id/vacations → 200 + عرض القائمة</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح.</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr"/>
+    </row>
+    <row r="21" ht="80" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>EM-052</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>حذف إجازة</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>حذف vacation record</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>إجازة موجودة</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط حذف بجانب الإجازة</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>DELETE /employees/:id/vacations/:vacationId → 204</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح.</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22" ht="80" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>EM-060</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>زر التقييمات والمراجعات</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>التنقل لصفحة ratings</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>1. اضغط (التقييمات والمراجعات) في PageHeader</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>1. التنقل لـ /ratings
+2. combobox اختيار ممارس
+3. اختيار ممارس → GET /employees/:id/ratings</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>نجح: combobox + empty state صحيحان.</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23" ht="80" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>EM-070</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Topbar user name</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>اسم المستخدم يظهر صحيحاً بدل ??</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>مستخدم admin</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>1. لاحظ أعلى يسار الصفحة</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>يعرض A — Admin — مدير العيادة (وليس ??)</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: الباك كان يرسل {name:Admin} والـ frontend يتوقع firstName/lastName. الآن يُقسم الاسم + fallback للإيميل.</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>P1-High</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: get-current-user.handler.ts + header.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="80" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>EM-080</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Branding endpoint لا يرمي 404</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>الصفحة تُحمَّل دون أخطاء branding في console</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>tenant بدون branding config</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح أي صفحة
+2. افتح console</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>GET /public/branding/:tenantId → 200 مع defaults (بدل 404)</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>نجح بعد الإصلاح: الـ handler كان يرمي NotFoundException، الآن يعيد defaults.</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P24" s="9" t="inlineStr">
+        <is>
+          <t>Fixed: get-branding.handler.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="80" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>EM-090</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Seed data نظيفة</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>عدم وجود سجلات ملوّثة (nameEn=General Checkup)</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>قاعدة بيانات dev</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح /employees</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>لا سجلات بأسماء خدمات في حقل الاسم</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>نجح: حُذفت 4 سجلات ملوّثة عبر prisma/clean-bad-employees.ts.</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N25" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26" ht="80" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>EM-100</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>BUG: التسعير المخصص للممارس</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>السعر/المدة/نوع الحجز للخدمة تُرسل لكن لا تُحفظ</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>ربط خدمة بتسعير مخصص</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>1. أنشئ ممارس
+2. اربط خدمة بـ 300 ر.س / 45 دق
+3. افتح detail</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>price=300, duration=45</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>detail يعرض (الأسعار: زيارة العيادة 300 / استشارة هاتفية —)</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>فشل: Schema EmployeeService لا تحتوي price/duration/types. يحتاج migration جديدة + model EmployeeServiceType. البيانات تُقبل بـ 201 لكن تُفقد.</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>P0-Critical</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P26" s="10" t="inlineStr">
+        <is>
+          <t>BLOCKED: migration drift في الـ repo يمنع schema changes. يحتاج قرار: reset أو fix-drift أو migration جديدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>EM-101</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>BUG: خانة الخبرة valuemax=0</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>spinbutton في فورم الإنشاء فيه max=0</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>فورم الإنشاء</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح create employee
+2. فحص خانة الخبرة</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>valuemax ≥ 100</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>فشل: الـ input HTML max=0. UX مربك لكن الـ form يقبل القيم عند الإرسال.</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>P3-Low</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N27" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P27" s="9" t="inlineStr">
+        <is>
+          <t>BUG: experience number input max attribute. Not blocking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="80" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>EM-102</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Employees (الممارسون)</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>BUG: GET /bookings 400</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>detail page يطلب bookings ويفشل</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>ممارس موجود</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>1. افتح detail
+2. لاحظ chart (الحجوزات حسب الحالة)</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>employeeId query param</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>GET /dashboard/bookings?employeeId=... → 200</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>فشل: 400 Bad Request. الـ charts لا تعمل.</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>P2-Medium</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="M28" s="9" t="inlineStr">
+        <is>
+          <t>Local dev</t>
+        </is>
+      </c>
+      <c r="N28" s="9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="O28" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="P28" s="10" t="inlineStr">
+        <is>
+          <t>BUG: bookings list DTO يرفض employeeId/fromDate/toDate params. خارج نطاق employees.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>